<commit_message>
Add hydrology data and resources
</commit_message>
<xml_diff>
--- a/Qp_Sokolovsky/Sokolovsky_Cầu_Phú_Kiểng.xlsx
+++ b/Qp_Sokolovsky/Sokolovsky_Cầu_Phú_Kiểng.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hiện trạng" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Xét BĐKH" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hiện trạng" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xét BĐKH" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -55,12 +57,18 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFDE7"/>
+        <bgColor rgb="00FFFDE7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -95,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -104,40 +112,56 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -505,10 +529,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H25"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -516,14 +540,19 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KẾT QUẢ TÍNH LŨ THEO XÔ-KÔ-LÔP-SKI - HIỆN TRẠNG - Cầu Phú Kiểng</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>I. THÔNG SỐ ĐẦU VÀO LƯU VỰC VÀ THỦY VĂN</t>
+          <t>I. THÔNG SỐ ĐẦU VÀO LƯU VỰC VÀ THỦY VĂN (ô vàng: số liệu nhập; ô còn lại: công thức)</t>
         </is>
       </c>
     </row>
@@ -558,7 +587,7 @@
           <t>Ls</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="4" t="n">
         <v>78.98</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -578,7 +607,7 @@
           <t>Ho</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="5" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -590,7 +619,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Vận tốc bình quân lớn nhất tại cửa ra</t>
+          <t>Vận tốc lớn nhất trên sườn dốc</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -598,7 +627,7 @@
           <t>Vmax</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -610,7 +639,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>H/S vận tốc truyền lũ tb lòng sông</t>
+          <t>H/S truyền lũ lòng sông</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -618,7 +647,7 @@
           <t>kv</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="6" t="n">
         <v>0.65</v>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -626,100 +655,97 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>H/S thời gian mưa rào</t>
+          <t>H/S thời gian theo vùng khí hậu</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>kt</t>
+          <t>km</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Hệ số dòng chảy lũ</t>
+          <t>H/S thời gian mưa rào</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>α</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>0.86</v>
+          <t>kt</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Hệ số hình dạng lũ</t>
+          <t>Hệ số dòng chảy lũ</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>f</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>0.7</v>
+          <t>α</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.86</v>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Hệ số triết giảm hồ ao, đầm lầy</t>
+          <t>Hệ số hình dạng lũ</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>δ</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>0.9005</v>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.7</v>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Thời gian tập trung nước trong sông</t>
+          <t>Hệ số triết giảm ao hồ, đầm lầy</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ts</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>16.88</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>giờ</t>
-        </is>
-      </c>
+          <t>δ</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0.9005</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Thời gian lũ lên</t>
+          <t>Thời gian tập trung nước trong sông</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>tl</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>16.88</v>
+          <t>ts</t>
+        </is>
+      </c>
+      <c r="C13" s="8">
+        <f>C4/(C7*C6*3.6)</f>
+        <v/>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -730,16 +756,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Thời gian mưa tính toán</t>
+          <t>Thời gian lũ lên</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>9.529999999999999</v>
+          <t>tl</t>
+        </is>
+      </c>
+      <c r="C14" s="8">
+        <f>C13</f>
+        <v/>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -750,284 +777,334 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Phân khu mưa rào</t>
+          <t>Thời gian mưa tính toán</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C15" s="8">
+        <f>C13*C8*C9</f>
+        <v/>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>giờ</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lưu lượng dòng chảy ngầm</t>
+          <t>Phân vùng mưa rào</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Qng</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>m³/s</t>
-        </is>
-      </c>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Tung độ ψ(T) (nội suy bảng tọa độ vùng R)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>ψ</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0.8371330484330484</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Hệ số triết giảm diện tích 1+0,001·F^0,8</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>ϑ</t>
+        </is>
+      </c>
+      <c r="C18" s="10">
+        <f>1+0.001*C3^0.8</f>
+        <v/>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>II. KẾT QUẢ TÍNH TOÁN THEO TẦN SUẤT THIẾT KẾ P (%)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Thông số tính toán</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Ký hiệu (Đơn vị)</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>1%</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>1.5%</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>4%</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Tần suất thiết kế</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>P (%)</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>1.0%</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>1.5%</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>4.0%</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>5.0%</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>10.0%</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Lượng mưa ngày thiết kế</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>H24p (mm)</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="n">
-        <v>396.8</v>
-      </c>
-      <c r="D21" s="12" t="n">
-        <v>369.2</v>
-      </c>
-      <c r="E21" s="12" t="n">
-        <v>304.1</v>
-      </c>
-      <c r="F21" s="12" t="n">
-        <v>289.6</v>
-      </c>
-      <c r="G21" s="12" t="n">
-        <v>245.1</v>
-      </c>
-      <c r="H21" s="12" t="n">
-        <v>140</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Tung độ đường cong lũ tích mưa</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>ψ(T)</t>
+          <t>Tần suất thiết kế</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>P (%)</t>
         </is>
       </c>
       <c r="C22" s="13" t="n">
-        <v>0.837</v>
+        <v>1</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>0.837</v>
+        <v>1.5</v>
       </c>
       <c r="E22" s="13" t="n">
-        <v>0.837</v>
+        <v>4</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.837</v>
+        <v>5</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.837</v>
+        <v>10</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>0.837</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Lượng mưa lũ thiết kế</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Htp (mm)</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="n">
-        <v>332.1</v>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>309.1</v>
-      </c>
-      <c r="E23" s="12" t="n">
-        <v>254.6</v>
-      </c>
-      <c r="F23" s="12" t="n">
-        <v>242.4</v>
-      </c>
-      <c r="G23" s="12" t="n">
-        <v>205.2</v>
-      </c>
-      <c r="H23" s="12" t="n">
-        <v>117.2</v>
+          <t>Lượng mưa ngày thiết kế</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>H24p (mm)</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>396.76</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>369.18</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>304.1</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>289.58</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>245.07</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>140.02</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Lượng mưa lũ thiết kế triết giảm</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
+          <t>Tung độ đường cong mưa rào</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>ψ(T)</t>
+        </is>
+      </c>
+      <c r="C24" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="D24" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="E24" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="F24" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="G24" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="H24" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Lượng mưa rào thiết kế</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Htp (mm)</t>
+        </is>
+      </c>
+      <c r="C25" s="16">
+        <f>C23*$C$17</f>
+        <v/>
+      </c>
+      <c r="D25" s="16">
+        <f>D23*$C$17</f>
+        <v/>
+      </c>
+      <c r="E25" s="16">
+        <f>E23*$C$17</f>
+        <v/>
+      </c>
+      <c r="F25" s="16">
+        <f>F23*$C$17</f>
+        <v/>
+      </c>
+      <c r="G25" s="16">
+        <f>G23*$C$17</f>
+        <v/>
+      </c>
+      <c r="H25" s="16">
+        <f>H23*$C$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Lượng mưa rào thiết kế triết giảm</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>H'tp (mm)</t>
         </is>
       </c>
-      <c r="C24" s="12" t="n">
-        <v>235.3</v>
-      </c>
-      <c r="D24" s="12" t="n">
-        <v>218.9</v>
-      </c>
-      <c r="E24" s="12" t="n">
-        <v>180.3</v>
-      </c>
-      <c r="F24" s="12" t="n">
-        <v>171.7</v>
-      </c>
-      <c r="G24" s="12" t="n">
-        <v>145.3</v>
-      </c>
-      <c r="H24" s="12" t="n">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="C26" s="16">
+        <f>C25/$C$18</f>
+        <v/>
+      </c>
+      <c r="D26" s="16">
+        <f>D25/$C$18</f>
+        <v/>
+      </c>
+      <c r="E26" s="16">
+        <f>E25/$C$18</f>
+        <v/>
+      </c>
+      <c r="F26" s="16">
+        <f>F25/$C$18</f>
+        <v/>
+      </c>
+      <c r="G26" s="16">
+        <f>G25/$C$18</f>
+        <v/>
+      </c>
+      <c r="H26" s="16">
+        <f>H25/$C$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Lưu lượng đỉnh lũ thiết kế</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>Qmax,p (m³/s)</t>
         </is>
       </c>
-      <c r="C25" s="15" t="n">
-        <v>3632</v>
-      </c>
-      <c r="D25" s="15" t="n">
-        <v>3361</v>
-      </c>
-      <c r="E25" s="15" t="n">
-        <v>2722</v>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>2579</v>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>2142</v>
-      </c>
-      <c r="H25" s="15" t="n">
-        <v>1110</v>
+      <c r="C27" s="19">
+        <f>0.278*$C$10*MAX(C26-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="D27" s="19">
+        <f>0.278*$C$10*MAX(D26-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="E27" s="19">
+        <f>0.278*$C$10*MAX(E26-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="F27" s="19">
+        <f>0.278*$C$10*MAX(F26-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="G27" s="19">
+        <f>0.278*$C$10*MAX(G26-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="H27" s="19">
+        <f>0.278*$C$10*MAX(H26-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t>Công thức: Qmax,p = 0,278·α·(H'tp − Ho)·f·F·δ / tl  (Q = 0 nếu H'tp ≤ Ho)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A18:H18"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1038,10 +1115,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H25"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1049,14 +1126,19 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KẾT QUẢ TÍNH LŨ THEO XÔ-KÔ-LÔP-SKI - XÉT BĐKH - Cầu Phú Kiểng</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>I. THÔNG SỐ ĐẦU VÀO LƯU VỰC VÀ THỦY VĂN</t>
+          <t>I. THÔNG SỐ ĐẦU VÀO LƯU VỰC VÀ THỦY VĂN (ô vàng: số liệu nhập; ô còn lại: công thức)</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1173,7 @@
           <t>Ls</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="4" t="n">
         <v>78.98</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1111,7 +1193,7 @@
           <t>Ho</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="5" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1123,7 +1205,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Vận tốc bình quân lớn nhất tại cửa ra</t>
+          <t>Vận tốc lớn nhất trên sườn dốc</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1131,7 +1213,7 @@
           <t>Vmax</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1143,7 +1225,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>H/S vận tốc truyền lũ tb lòng sông</t>
+          <t>H/S truyền lũ lòng sông</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1151,7 +1233,7 @@
           <t>kv</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="6" t="n">
         <v>0.65</v>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -1159,100 +1241,97 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>H/S thời gian mưa rào</t>
+          <t>H/S thời gian theo vùng khí hậu</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>kt</t>
+          <t>km</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Hệ số dòng chảy lũ</t>
+          <t>H/S thời gian mưa rào</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>α</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>0.86</v>
+          <t>kt</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Hệ số hình dạng lũ</t>
+          <t>Hệ số dòng chảy lũ</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>f</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>0.7</v>
+          <t>α</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.86</v>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Hệ số triết giảm hồ ao, đầm lầy</t>
+          <t>Hệ số hình dạng lũ</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>δ</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>0.9005</v>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.7</v>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Thời gian tập trung nước trong sông</t>
+          <t>Hệ số triết giảm ao hồ, đầm lầy</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>ts</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>16.88</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>giờ</t>
-        </is>
-      </c>
+          <t>δ</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0.9005</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Thời gian lũ lên</t>
+          <t>Thời gian tập trung nước trong sông</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>tl</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>16.88</v>
+          <t>ts</t>
+        </is>
+      </c>
+      <c r="C13" s="8">
+        <f>C4/(C7*C6*3.6)</f>
+        <v/>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -1263,16 +1342,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Thời gian mưa tính toán</t>
+          <t>Thời gian lũ lên</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>9.529999999999999</v>
+          <t>tl</t>
+        </is>
+      </c>
+      <c r="C14" s="8">
+        <f>C13</f>
+        <v/>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -1283,284 +1363,400 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Phân khu mưa rào</t>
+          <t>Thời gian mưa tính toán</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="C15" s="8">
+        <f>C13*C8*C9</f>
+        <v/>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>giờ</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lưu lượng dòng chảy ngầm</t>
+          <t>Phân vùng mưa rào</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Qng</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>m³/s</t>
-        </is>
-      </c>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Tung độ ψ(T) (nội suy bảng tọa độ vùng R)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>ψ</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0.8371330484330484</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>III. KẾT QUẢ TÍNH TOÁN THEO TẦN SUẤT THIẾT KẾ P (%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Hệ số triết giảm diện tích 1+0,001·F^0,8</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>ϑ</t>
+        </is>
+      </c>
+      <c r="C18" s="10">
+        <f>1+0.001*C3^0.8</f>
+        <v/>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>II. KẾT QUẢ TÍNH TOÁN THEO TẦN SUẤT THIẾT KẾ P (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Thông số tính toán</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Ký hiệu (Đơn vị)</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>1%</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>1.5%</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>4%</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Tần suất thiết kế</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>P (%)</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>1.0%</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>1.5%</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>4.0%</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>5.0%</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>10.0%</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Lượng mưa ngày thiết kế</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>H24p (mm)</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="n">
-        <v>450.3</v>
-      </c>
-      <c r="D21" s="12" t="n">
-        <v>419</v>
-      </c>
-      <c r="E21" s="12" t="n">
-        <v>345.2</v>
-      </c>
-      <c r="F21" s="12" t="n">
-        <v>328.7</v>
-      </c>
-      <c r="G21" s="12" t="n">
-        <v>278.2</v>
-      </c>
-      <c r="H21" s="12" t="n">
-        <v>158.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Tung độ đường cong lũ tích mưa</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>ψ(T)</t>
+          <t>Tần suất thiết kế</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>P (%)</t>
         </is>
       </c>
       <c r="C22" s="13" t="n">
-        <v>0.837</v>
+        <v>1</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>0.837</v>
+        <v>1.5</v>
       </c>
       <c r="E22" s="13" t="n">
-        <v>0.837</v>
+        <v>4</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.837</v>
+        <v>5</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.837</v>
+        <v>10</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>0.837</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Lượng mưa lũ thiết kế</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Htp (mm)</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="n">
-        <v>377</v>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>350.8</v>
-      </c>
-      <c r="E23" s="12" t="n">
-        <v>288.9</v>
-      </c>
-      <c r="F23" s="12" t="n">
-        <v>275.1</v>
-      </c>
-      <c r="G23" s="12" t="n">
-        <v>232.9</v>
-      </c>
-      <c r="H23" s="12" t="n">
-        <v>133</v>
+          <t>Lượng mưa ngày (số liệu gốc)</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>H24p gốc (mm)</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>396.76</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>369.18</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>304.1</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>289.58</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>245.07</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>140.02</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Lượng mưa lũ thiết kế triết giảm</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
+          <t>Hệ số biến đổi khí hậu</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Kbđkh</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="D24" s="21" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="E24" s="21" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="F24" s="21" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="G24" s="21" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="H24" s="21" t="n">
+        <v>1.135</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Lượng mưa ngày thiết kế xét BĐKH</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>H24p (mm)</t>
+        </is>
+      </c>
+      <c r="C25" s="16">
+        <f>C23*C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="16">
+        <f>D23*D24</f>
+        <v/>
+      </c>
+      <c r="E25" s="16">
+        <f>E23*E24</f>
+        <v/>
+      </c>
+      <c r="F25" s="16">
+        <f>F23*F24</f>
+        <v/>
+      </c>
+      <c r="G25" s="16">
+        <f>G23*G24</f>
+        <v/>
+      </c>
+      <c r="H25" s="16">
+        <f>H23*H24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Tung độ đường cong mưa rào</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>ψ(T)</t>
+        </is>
+      </c>
+      <c r="C26" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="D26" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="E26" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="F26" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="G26" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+      <c r="H26" s="15">
+        <f>$C$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Lượng mưa rào thiết kế</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Htp (mm)</t>
+        </is>
+      </c>
+      <c r="C27" s="16">
+        <f>C25*$C$17</f>
+        <v/>
+      </c>
+      <c r="D27" s="16">
+        <f>D25*$C$17</f>
+        <v/>
+      </c>
+      <c r="E27" s="16">
+        <f>E25*$C$17</f>
+        <v/>
+      </c>
+      <c r="F27" s="16">
+        <f>F25*$C$17</f>
+        <v/>
+      </c>
+      <c r="G27" s="16">
+        <f>G25*$C$17</f>
+        <v/>
+      </c>
+      <c r="H27" s="16">
+        <f>H25*$C$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Lượng mưa rào thiết kế triết giảm</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>H'tp (mm)</t>
         </is>
       </c>
-      <c r="C24" s="12" t="n">
-        <v>267</v>
-      </c>
-      <c r="D24" s="12" t="n">
-        <v>248.5</v>
-      </c>
-      <c r="E24" s="12" t="n">
-        <v>204.7</v>
-      </c>
-      <c r="F24" s="12" t="n">
-        <v>194.9</v>
-      </c>
-      <c r="G24" s="12" t="n">
-        <v>164.9</v>
-      </c>
-      <c r="H24" s="12" t="n">
-        <v>94.2</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="C28" s="16">
+        <f>C27/$C$18</f>
+        <v/>
+      </c>
+      <c r="D28" s="16">
+        <f>D27/$C$18</f>
+        <v/>
+      </c>
+      <c r="E28" s="16">
+        <f>E27/$C$18</f>
+        <v/>
+      </c>
+      <c r="F28" s="16">
+        <f>F27/$C$18</f>
+        <v/>
+      </c>
+      <c r="G28" s="16">
+        <f>G27/$C$18</f>
+        <v/>
+      </c>
+      <c r="H28" s="16">
+        <f>H27/$C$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Lưu lượng đỉnh lũ thiết kế</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Qmax,p (m³/s)</t>
         </is>
       </c>
-      <c r="C25" s="15" t="n">
-        <v>4158</v>
-      </c>
-      <c r="D25" s="15" t="n">
-        <v>3851</v>
-      </c>
-      <c r="E25" s="15" t="n">
-        <v>3125</v>
-      </c>
-      <c r="F25" s="15" t="n">
-        <v>2963</v>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>2467</v>
-      </c>
-      <c r="H25" s="15" t="n">
-        <v>1296</v>
+      <c r="C29" s="19">
+        <f>0.278*$C$10*MAX(C28-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="D29" s="19">
+        <f>0.278*$C$10*MAX(D28-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="E29" s="19">
+        <f>0.278*$C$10*MAX(E28-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="F29" s="19">
+        <f>0.278*$C$10*MAX(F28-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="G29" s="19">
+        <f>0.278*$C$10*MAX(G28-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+      <c r="H29" s="19">
+        <f>0.278*$C$10*MAX(H28-$C$5,0)*$C$11*$C$3*$C$12/$C$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>Công thức: Qmax,p = 0,278·α·(H'tp − Ho)·f·F·δ / tl  (Q = 0 nếu H'tp ≤ Ho)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A18:H18"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>